<commit_message>
Re-underwrite 8 OM-on-file deals from the OM rent rolls and expense statements; rebuild master and Shawn Mangoli pages
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/02-2001-penmar-ave.xlsx
+++ b/files/02-2001-penmar-ave.xlsx
@@ -8,17 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AE3D756-405B-4792-A6DA-58C123E583EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3CF6438-C08C-47BD-AC5E-A50A5340BDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7A4689AD-2101-4028-99BD-966916D0152F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E2BABCE3-DF98-4F8E-954C-23F2036EA389}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
     <sheet name="02 2001 Penmar Ave" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'02 2001 Penmar Ave'!$A$1:$N$78</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="144">
   <si>
     <t>LAAA UNDERWRITING BENCHMARKS (edit here; every deal tab reads these)</t>
   </si>
@@ -195,10 +192,10 @@
     <t>LoopNet listing</t>
   </si>
   <si>
-    <t>Data pulled 9/17/2026 from LoopNet public listing</t>
-  </si>
-  <si>
-    <t>NOTE: New listing 9/15/26, remodeled</t>
+    <t>Data pulled 9/17/2026 from LoopNet public listing + rent roll and expenses read from the listing broker's OM (RE/MAX, Taksa Investment Group, undated, rent roll May 2026)</t>
+  </si>
+  <si>
+    <t>NOTE: New listing 9/15/26, remodeled | OM: OM date not printed; latest move-in date on rent roll is 5/4/26 so the roll is mid-2026 or later.; Rent roll page text layer was scrambled; current rents read from the rendered page image. Unit-by-unit sum $37,286/mo vs OM total $37,283 ($3 rounding diff, within 1%); annual $447,401 per OM.; Current | OM: OM date not printed; latest move-in date on rent roll is 5/4/26 so the roll is mid-2026 or later.; Rent roll page text layer was scrambled; current rents read from the rendered page image. Unit-by-unit sum $37,286/mo vs OM total $37,283 ($3 rounding diff, within 1%); annual $447,401 per OM.; Current</t>
   </si>
   <si>
     <t>PROPERTY</t>
@@ -300,19 +297,22 @@
     <t>Rent source</t>
   </si>
   <si>
-    <t>Studio  (~450 SF)</t>
-  </si>
-  <si>
-    <t>Allocated from published GRM (price / GRM) using LAAA bed weights</t>
-  </si>
-  <si>
-    <t>1 Bd / 1 Ba  (~625 SF)</t>
-  </si>
-  <si>
-    <t>2 Bd / 1 Ba  (~758 SF)</t>
-  </si>
-  <si>
-    <t>2 Bd / 2 Ba  (~758 SF)</t>
+    <t>Studio  (~450 SF)  [Units 1, 11; rents $2,248 and $2,038; market $2,300]</t>
+  </si>
+  <si>
+    <t>OM rent roll, current in-place rents (OM undated, rent roll May 2026)</t>
+  </si>
+  <si>
+    <t>1 Bd / 1 Ba  (~625 SF)  [Units 3-6; rents $1,205 / $3,073 / $1,309 / $3,153 (two lega]</t>
+  </si>
+  <si>
+    <t>2 Bd / 1 Ba  (~758 SF)  [Units 7-10 at 800 SF plus unit 13 attached ADU at 588 SF; re]</t>
+  </si>
+  <si>
+    <t>2 Bd / 2 Ba  (~694 SF)  [Unit 2 (800 SF, $3,348) and unit 12 attached ADU (588 SF, $3]</t>
+  </si>
+  <si>
+    <t>2 Bd / 2 Ba Two-Story Townhome (detached ADU)  (~887 SF)  [Unit 14 detached ADU; market $3,800]</t>
   </si>
   <si>
     <t>Total / weighted avg</t>
@@ -333,7 +333,7 @@
     <t>Scheduled gross rent</t>
   </si>
   <si>
-    <t>OM column: price / published GRM</t>
+    <t>OM column: OM stated current scheduled rent (OM undated, rent roll May 2026); LAAA column: OM rent roll by unit type</t>
   </si>
   <si>
     <t>Other income (laundry, parking, RUBS)</t>
@@ -345,7 +345,7 @@
     <t>Vacancy &amp; credit loss</t>
   </si>
   <si>
-    <t>OM 3.0% (OM figure if extracted, else 3% assumed); LAAA per Assumptions</t>
+    <t>OM 3.0%; LAAA per Assumptions</t>
   </si>
   <si>
     <t>Effective gross income</t>
@@ -390,7 +390,7 @@
     <t>Utilities (water/sewer/trash/common electric &amp; gas)</t>
   </si>
   <si>
-    <t>per unit, by city</t>
+    <t>per unit, by city; OM utilities + water/sewer + gas/electric + trash combined</t>
   </si>
   <si>
     <t>Contract services (landscape, pest, cleaning)</t>
@@ -399,10 +399,10 @@
     <t>per unit</t>
   </si>
   <si>
-    <t>Admin / legal / licenses / rent registration</t>
-  </si>
-  <si>
-    <t>per unit; OM "other" items land here</t>
+    <t>Admin / legal / licenses / rent registration / other OM items</t>
+  </si>
+  <si>
+    <t>OM other items: Miscellaneous 2,500</t>
   </si>
   <si>
     <t>Replacement reserves</t>
@@ -411,7 +411,7 @@
     <t>Total operating expenses</t>
   </si>
   <si>
-    <t>OM line items not published. OM total IMPLIED = OM EGI - (price x published cap)</t>
+    <t>OM line items from OM (OM undated, rent roll May 2026); basis: OM 'Current' column of Estimated Expenses (page 17); broker estimates per OM note ('estimated only, based partly on industry standards'). Taxes = 1.175% of list price (reassessed at sale, not seller actual). Management 4% of scheduled rent. R&amp;M assumed $500/unit/yr. Utilities is a single $12,000 line (water/gas/electric not split). Pro forma total is $124,030 (only management changes).; OM total 119,654</t>
   </si>
   <si>
     <t>Expenses per unit</t>
@@ -427,6 +427,9 @@
   </si>
   <si>
     <t>Net operating income</t>
+  </si>
+  <si>
+    <t>OM states NOI 316,125 / cap 6.2</t>
   </si>
   <si>
     <t>Cap rate on asking price</t>
@@ -475,12 +478,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$#,##0;\(\$#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0;\(&quot;$&quot;#,##0\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -528,6 +532,7 @@
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -536,8 +541,21 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -565,7 +583,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF9E5"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -601,7 +620,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -625,12 +644,15 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -663,7 +685,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{835F6268-B399-4172-A1D8-4C166A3AC7AB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C665A5E-A5CD-42B4-9617-4D7714C3C217}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -974,7 +996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DF668F-136D-4471-9061-C68E341DE64F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE24FF7D-5CF0-45D4-80B2-C836386C6948}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1343,11 +1365,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7470BF3A-8C8F-4664-8A7B-7749305ED48E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA685BAD-5649-4B62-AEBC-769DA7D7186A}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -1577,17 +1599,17 @@
         <v>2</v>
       </c>
       <c r="C30" s="21">
-        <v>1618</v>
-      </c>
-      <c r="D30" s="8">
+        <v>2143</v>
+      </c>
+      <c r="D30" s="22">
         <f>B30*C30</f>
-        <v>3236</v>
-      </c>
-      <c r="E30" s="8">
+        <v>4286</v>
+      </c>
+      <c r="E30" s="22">
         <f>D30*12</f>
-        <v>38832</v>
-      </c>
-      <c r="F30" s="2" t="s">
+        <v>51432</v>
+      </c>
+      <c r="F30" s="23" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1599,17 +1621,17 @@
         <v>4</v>
       </c>
       <c r="C31" s="21">
-        <v>2311</v>
-      </c>
-      <c r="D31" s="8">
+        <v>2185</v>
+      </c>
+      <c r="D31" s="22">
         <f>B31*C31</f>
-        <v>9244</v>
-      </c>
-      <c r="E31" s="8">
+        <v>8740</v>
+      </c>
+      <c r="E31" s="22">
         <f>D31*12</f>
-        <v>110928</v>
-      </c>
-      <c r="F31" s="2" t="s">
+        <v>104880</v>
+      </c>
+      <c r="F31" s="23" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1621,17 +1643,17 @@
         <v>5</v>
       </c>
       <c r="C32" s="21">
-        <v>3120</v>
-      </c>
-      <c r="D32" s="8">
+        <v>2770</v>
+      </c>
+      <c r="D32" s="22">
         <f>B32*C32</f>
-        <v>15600</v>
-      </c>
-      <c r="E32" s="8">
+        <v>13850</v>
+      </c>
+      <c r="E32" s="22">
         <f>D32*12</f>
-        <v>187200</v>
-      </c>
-      <c r="F32" s="2" t="s">
+        <v>166200</v>
+      </c>
+      <c r="F32" s="23" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1640,574 +1662,612 @@
         <v>89</v>
       </c>
       <c r="B33" s="15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" s="21">
-        <v>3120</v>
-      </c>
-      <c r="D33" s="8">
+        <v>3306</v>
+      </c>
+      <c r="D33" s="22">
         <f>B33*C33</f>
-        <v>9360</v>
-      </c>
-      <c r="E33" s="8">
+        <v>6612</v>
+      </c>
+      <c r="E33" s="22">
         <f>D33*12</f>
-        <v>112320</v>
-      </c>
-      <c r="F33" s="2" t="s">
+        <v>79344</v>
+      </c>
+      <c r="F33" s="23" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="22" t="s">
+      <c r="A34" t="s">
         <v>90</v>
       </c>
-      <c r="B34" s="23">
-        <f>SUM(B30:B33)</f>
+      <c r="B34" s="15">
+        <v>1</v>
+      </c>
+      <c r="C34" s="21">
+        <v>3798</v>
+      </c>
+      <c r="D34" s="22">
+        <f>B34*C34</f>
+        <v>3798</v>
+      </c>
+      <c r="E34" s="22">
+        <f>D34*12</f>
+        <v>45576</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="B35" s="25">
+        <f>SUM(B30:B34)</f>
         <v>14</v>
       </c>
-      <c r="C34" s="24">
-        <f>IFERROR(D34/B34,"")</f>
-        <v>2674.2857142857142</v>
-      </c>
-      <c r="D34" s="24">
-        <f>SUM(D30:D33)</f>
-        <v>37440</v>
-      </c>
-      <c r="E34" s="24">
-        <f>SUM(E30:E33)</f>
-        <v>449280</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
+      <c r="C35" s="26">
+        <f>IFERROR(D35/B35,"")</f>
+        <v>2663.2857142857142</v>
+      </c>
+      <c r="D35" s="26">
+        <f>SUM(D30:D34)</f>
+        <v>37286</v>
+      </c>
+      <c r="E35" s="26">
+        <f>SUM(E30:E34)</f>
+        <v>447432</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="25"/>
-      <c r="B37" s="25" t="s">
+      <c r="A37" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="25" t="s">
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="27"/>
+      <c r="B38" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="D37" s="25"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25" t="s">
+      <c r="C38" s="27" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="D38" s="27"/>
+      <c r="E38" s="27"/>
+      <c r="F38" s="27" t="s">
         <v>95</v>
-      </c>
-      <c r="B38" s="8">
-        <v>449294.53262786602</v>
-      </c>
-      <c r="C38" s="8">
-        <f>E34</f>
-        <v>449280</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>96</v>
+      </c>
+      <c r="B39" s="22">
+        <v>447401</v>
+      </c>
+      <c r="C39" s="8">
+        <f>E35</f>
+        <v>447432</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B39" s="8">
-        <v>0</v>
-      </c>
-      <c r="C39" s="4">
-        <v>0</v>
-      </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
+      <c r="A40" t="s">
         <v>98</v>
       </c>
       <c r="B40" s="8">
-        <f>B38+B39</f>
-        <v>449294.53262786602</v>
-      </c>
-      <c r="C40" s="8">
-        <f>C38+C39</f>
-        <v>449280</v>
+        <v>1800</v>
+      </c>
+      <c r="C40" s="4">
+        <v>1800</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="A41" s="24" t="s">
         <v>99</v>
       </c>
       <c r="B41" s="8">
-        <f>-B38*0.03</f>
-        <v>-13478.835978835979</v>
+        <f>B39+B40</f>
+        <v>449201</v>
       </c>
       <c r="C41" s="8">
-        <f>-C38*Assumptions!$B$3</f>
-        <v>-13478.4</v>
-      </c>
-      <c r="F41" s="2" t="s">
+        <f>C39+C40</f>
+        <v>449232</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="22" t="s">
+      <c r="B42" s="8">
+        <f>-B39*0.03</f>
+        <v>-13422.029999999999</v>
+      </c>
+      <c r="C42" s="8">
+        <f>-C39*Assumptions!$B$3</f>
+        <v>-13422.96</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B42" s="24">
-        <f>B40+B41</f>
-        <v>435815.69664903003</v>
-      </c>
-      <c r="C42" s="24">
-        <f>C40+C41</f>
-        <v>435801.59999999998</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="13" t="s">
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
+      <c r="B43" s="26">
+        <f>B41+B42</f>
+        <v>435778.97</v>
+      </c>
+      <c r="C43" s="26">
+        <f>C41+C42</f>
+        <v>435809.04</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
+      <c r="A45" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C45" s="25" t="s">
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D45" s="25" t="s">
+      <c r="B46" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="E45" s="25" t="s">
+      <c r="C46" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="F45" s="25" t="s">
+      <c r="D46" s="27" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="E46" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8">
+      <c r="F46" s="27" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>107</v>
+      </c>
+      <c r="B47" s="22">
+        <v>59866</v>
+      </c>
+      <c r="C47" s="8">
         <f>B22*Assumptions!$B$15</f>
         <v>63687.5</v>
       </c>
-      <c r="D46" s="26">
-        <f>C46</f>
+      <c r="D47" s="28">
+        <f>C47</f>
         <v>63687.5</v>
       </c>
-      <c r="E46" s="8" t="str">
-        <f t="shared" ref="E46:E54" si="0">IF(ISNUMBER(B46),D46-B46,"")</f>
-        <v/>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="E47" s="8">
+        <f t="shared" ref="E47:E55" si="0">IF(ISNUMBER(B47),D47-B47,"")</f>
+        <v>3821.5</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8">
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>109</v>
+      </c>
+      <c r="B48" s="22">
+        <v>12392</v>
+      </c>
+      <c r="C48" s="8">
         <f>B7*Assumptions!$B$5+B8*Assumptions!$B$6</f>
         <v>12332</v>
       </c>
-      <c r="D47" s="26">
-        <f t="shared" ref="D47:D53" si="1">IF(ISNUMBER(B47),MAX(B47,C47),C47)</f>
-        <v>12332</v>
-      </c>
-      <c r="E47" s="8" t="str">
+      <c r="D48" s="28">
+        <f t="shared" ref="D48:D54" si="1">IF(ISNUMBER(B48),MAX(B48,C48),C48)</f>
+        <v>12392</v>
+      </c>
+      <c r="E48" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>111</v>
+      </c>
+      <c r="B49" s="22">
+        <v>17896</v>
+      </c>
+      <c r="C49" s="8">
+        <f>C43*Assumptions!$B$4</f>
+        <v>21790.452000000001</v>
+      </c>
+      <c r="D49" s="28">
+        <f t="shared" si="1"/>
+        <v>21790.452000000001</v>
+      </c>
+      <c r="E49" s="8">
+        <f t="shared" si="0"/>
+        <v>3894.4520000000011</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>113</v>
+      </c>
+      <c r="B50" s="22">
+        <v>7000</v>
+      </c>
+      <c r="C50" s="8">
+        <f>B7*Assumptions!$B$7</f>
+        <v>16800</v>
+      </c>
+      <c r="D50" s="28">
+        <f t="shared" si="1"/>
+        <v>16800</v>
+      </c>
+      <c r="E50" s="8">
+        <f t="shared" si="0"/>
+        <v>9800</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>115</v>
+      </c>
+      <c r="B51" s="22">
+        <v>15600</v>
+      </c>
+      <c r="C51" s="8">
+        <f>B7*Assumptions!$B$9</f>
+        <v>21000</v>
+      </c>
+      <c r="D51" s="28">
+        <f t="shared" si="1"/>
+        <v>21000</v>
+      </c>
+      <c r="E51" s="8">
+        <f t="shared" si="0"/>
+        <v>5400</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>117</v>
+      </c>
+      <c r="B52" s="22">
+        <v>4400</v>
+      </c>
+      <c r="C52" s="8">
+        <f>B7*Assumptions!$B$12</f>
+        <v>5600</v>
+      </c>
+      <c r="D52" s="28">
+        <f t="shared" si="1"/>
+        <v>5600</v>
+      </c>
+      <c r="E52" s="8">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>119</v>
+      </c>
+      <c r="B53" s="22">
+        <v>2500</v>
+      </c>
+      <c r="C53" s="8">
+        <f>B7*Assumptions!$B$13</f>
+        <v>3500</v>
+      </c>
+      <c r="D53" s="28">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
+      <c r="E53" s="8">
+        <f t="shared" si="0"/>
+        <v>1000</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>121</v>
+      </c>
+      <c r="B54" s="22"/>
+      <c r="C54" s="8">
+        <f>B7*Assumptions!$B$14</f>
+        <v>4200</v>
+      </c>
+      <c r="D54" s="28">
+        <f t="shared" si="1"/>
+        <v>4200</v>
+      </c>
+      <c r="E54" s="8" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="F47" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>110</v>
-      </c>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8">
-        <f>C42*Assumptions!$B$4</f>
-        <v>21790.080000000002</v>
-      </c>
-      <c r="D48" s="26">
-        <f t="shared" si="1"/>
-        <v>21790.080000000002</v>
-      </c>
-      <c r="E48" s="8" t="str">
+      <c r="F54" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B55" s="26">
+        <f>SUM(B47:B54)</f>
+        <v>119654</v>
+      </c>
+      <c r="C55" s="26">
+        <f>SUM(C47:C54)</f>
+        <v>148909.95199999999</v>
+      </c>
+      <c r="D55" s="26">
+        <f>SUM(D47:D54)</f>
+        <v>148969.95199999999</v>
+      </c>
+      <c r="E55" s="26">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>112</v>
-      </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8">
-        <f>B7*Assumptions!$B$7</f>
-        <v>16800</v>
-      </c>
-      <c r="D49" s="26">
-        <f t="shared" si="1"/>
-        <v>16800</v>
-      </c>
-      <c r="E49" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>114</v>
-      </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8">
-        <f>B7*Assumptions!$B$9</f>
-        <v>21000</v>
-      </c>
-      <c r="D50" s="26">
-        <f t="shared" si="1"/>
-        <v>21000</v>
-      </c>
-      <c r="E50" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>116</v>
-      </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8">
-        <f>B7*Assumptions!$B$12</f>
-        <v>5600</v>
-      </c>
-      <c r="D51" s="26">
-        <f t="shared" si="1"/>
-        <v>5600</v>
-      </c>
-      <c r="E51" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>118</v>
-      </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8">
-        <f>B7*Assumptions!$B$13</f>
-        <v>3500</v>
-      </c>
-      <c r="D52" s="26">
-        <f t="shared" si="1"/>
-        <v>3500</v>
-      </c>
-      <c r="E52" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>120</v>
-      </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8">
-        <f>B7*Assumptions!$B$14</f>
-        <v>4200</v>
-      </c>
-      <c r="D53" s="26">
-        <f t="shared" si="1"/>
-        <v>4200</v>
-      </c>
-      <c r="E53" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="B54" s="24">
-        <f>B42-B22*B25</f>
-        <v>119925.69664903003</v>
-      </c>
-      <c r="C54" s="24">
-        <f>SUM(C46:C53)</f>
-        <v>148909.58000000002</v>
-      </c>
-      <c r="D54" s="24">
-        <f>SUM(D46:D53)</f>
-        <v>148909.58000000002</v>
-      </c>
-      <c r="E54" s="24">
-        <f t="shared" si="0"/>
-        <v>28983.883350969991</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+        <v>29315.95199999999</v>
+      </c>
+      <c r="F55" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="B55" s="8">
-        <f>IFERROR(B54/B7,"")</f>
-        <v>8566.1211892164301</v>
-      </c>
-      <c r="C55" s="8">
-        <f>IFERROR(C54/B7,"")</f>
-        <v>10636.398571428572</v>
-      </c>
-      <c r="D55" s="8">
-        <f>IFERROR(D54/B7,"")</f>
-        <v>10636.398571428572</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>124</v>
       </c>
-      <c r="B56" s="18">
-        <f>IFERROR(B54/B42,"")</f>
-        <v>0.27517525773195883</v>
-      </c>
-      <c r="C56" s="18">
-        <f>IFERROR(C54/C42,"")</f>
-        <v>0.34169121912356454</v>
-      </c>
-      <c r="D56" s="18">
-        <f>IF(C38&gt;0,IFERROR(D54/C42,""),"")</f>
-        <v>0.34169121912356454</v>
+      <c r="B56" s="8">
+        <f>IFERROR(B55/B7,"")</f>
+        <v>8546.7142857142862</v>
+      </c>
+      <c r="C56" s="8">
+        <f>IFERROR(C55/B7,"")</f>
+        <v>10636.425142857142</v>
+      </c>
+      <c r="D56" s="8">
+        <f>IFERROR(D55/B7,"")</f>
+        <v>10640.710857142856</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="22" t="s">
+      <c r="A57" t="s">
         <v>125</v>
       </c>
-      <c r="B57" s="12" t="str">
-        <f>IF(ISNUMBER(B54),IF(D54&gt;B54*(1+Assumptions!$B$24),"OM EXPENSES LIGHT","OM expenses reasonable"),"OM expenses not published")</f>
+      <c r="B57" s="18">
+        <f>IFERROR(B55/B43,"")</f>
+        <v>0.2745749754743787</v>
+      </c>
+      <c r="C57" s="18">
+        <f>IFERROR(C55/C43,"")</f>
+        <v>0.34168623945937421</v>
+      </c>
+      <c r="D57" s="18">
+        <f>IF(C39&gt;0,IFERROR(D55/C43,""),"")</f>
+        <v>0.34182391443738752</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B58" s="29" t="str">
+        <f>IF(ISNUMBER(B55),IF(D55&gt;B55*(1+Assumptions!$B$24),"OM EXPENSES LIGHT","OM expenses reasonable"),"OM expenses not published")</f>
         <v>OM EXPENSES LIGHT</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="B59" s="14"/>
-      <c r="C59" s="14"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="14"/>
-    </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="25"/>
-      <c r="B60" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="C60" s="25" t="s">
+      <c r="A60" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B60" s="14"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="27"/>
+      <c r="B61" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="D60" s="25"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="25" t="s">
+      <c r="C61" s="27" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="B61" s="24">
-        <f>B42-B54</f>
-        <v>315890</v>
-      </c>
-      <c r="C61" s="24">
-        <f>IF(C38&gt;0,C42-D54,"")</f>
-        <v>286892.01999999996</v>
+      <c r="D61" s="27"/>
+      <c r="E61" s="27"/>
+      <c r="F61" s="27" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="22" t="s">
+      <c r="A62" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="B62" s="18">
-        <f>IFERROR(B61/B22,"")</f>
-        <v>6.2E-2</v>
-      </c>
-      <c r="C62" s="18">
-        <f>IF(C61="","",IFERROR(C61/B22,""))</f>
-        <v>5.630854170755642E-2</v>
-      </c>
-      <c r="F62" s="2" t="s">
+      <c r="B62" s="26">
+        <f>B43-B55</f>
+        <v>316124.96999999997</v>
+      </c>
+      <c r="C62" s="26">
+        <f>IF(C39&gt;0,C43-D55,"")</f>
+        <v>286839.08799999999</v>
+      </c>
+      <c r="F62" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+      <c r="A63" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="B63" s="19">
-        <f>IFERROR(B22/B38,"")</f>
-        <v>11.339999999999998</v>
-      </c>
-      <c r="C63" s="19">
-        <f>IF(C38&gt;0,IFERROR(B22/C38,""),"")</f>
-        <v>11.340366809116809</v>
+      <c r="B63" s="18">
+        <f>IFERROR(B62/B22,"")</f>
+        <v>6.204611776251226E-2</v>
+      </c>
+      <c r="C63" s="18">
+        <f>IF(C62="","",IFERROR(C62/B22,""))</f>
+        <v>5.6298152698724235E-2</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>131</v>
-      </c>
-      <c r="B64" s="8">
-        <f>IFERROR(B61/B7,"")</f>
-        <v>22563.571428571428</v>
-      </c>
-      <c r="C64" s="8">
-        <f>IF(C61="","",IFERROR(C61/B7,""))</f>
-        <v>20492.287142857142</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B66" s="14"/>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
-      <c r="F66" s="14"/>
+      <c r="B64" s="19">
+        <f>IFERROR(B22/B39,"")</f>
+        <v>11.387994215480072</v>
+      </c>
+      <c r="C64" s="19">
+        <f>IF(C39&gt;0,IFERROR(B22/C39,""),"")</f>
+        <v>11.387205206601227</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>133</v>
+      </c>
+      <c r="B65" s="8">
+        <f>IFERROR(B62/B7,"")</f>
+        <v>22580.355</v>
+      </c>
+      <c r="C65" s="8">
+        <f>IF(C62="","",IFERROR(C62/B7,""))</f>
+        <v>20488.506285714284</v>
+      </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>133</v>
-      </c>
-      <c r="B67" s="8">
+      <c r="A67" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B67" s="14"/>
+      <c r="C67" s="14"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="14"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>135</v>
+      </c>
+      <c r="B68" s="8">
         <f>IFERROR(B22*Assumptions!$B$20,"")</f>
         <v>3057000</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>134</v>
-      </c>
-      <c r="B68" s="8">
-        <f>IF(C61="","",IFERROR(PV(Assumptions!$B$22/12,Assumptions!$B$23*12,-C61/Assumptions!$B$21/12),""))</f>
-        <v>3106318.0715792128</v>
-      </c>
-    </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="22" t="s">
-        <v>135</v>
+      <c r="A69" t="s">
+        <v>136</v>
       </c>
       <c r="B69" s="8">
-        <f>IFERROR(MIN(B67,B68),"")</f>
+        <f>IF(C62="","",IFERROR(PV(Assumptions!$B$22/12,Assumptions!$B$23*12,-C62/Assumptions!$B$21/12),""))</f>
+        <v>3105744.9513224531</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="B70" s="8">
+        <f>IFERROR(MIN(B68,B69),"")</f>
         <v>3057000</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>136</v>
-      </c>
-      <c r="B70" s="8">
-        <f>IFERROR(B22-B69,"")</f>
-        <v>2038000</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B71" s="8">
-        <f>IFERROR(-PMT(Assumptions!$B$22/12,Assumptions!$B$23*12,B69)*12,"")</f>
-        <v>225869.69780441746</v>
+        <f>IFERROR(B22-B70,"")</f>
+        <v>2038000</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>138</v>
-      </c>
-      <c r="B72" s="19">
-        <f>IFERROR(C61/B71,"")</f>
-        <v>1.2701660416990608</v>
+        <v>139</v>
+      </c>
+      <c r="B72" s="8">
+        <f>IFERROR(-PMT(Assumptions!$B$22/12,Assumptions!$B$23*12,B70)*12,"")</f>
+        <v>225869.69780441746</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>139</v>
-      </c>
-      <c r="B73" s="8">
-        <f>IFERROR(C61-B71,"")</f>
-        <v>61022.322195582499</v>
+        <v>140</v>
+      </c>
+      <c r="B73" s="19">
+        <f>IFERROR(C62/B72,"")</f>
+        <v>1.269931694194661</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>140</v>
-      </c>
-      <c r="B74" s="18">
-        <f>IFERROR(B73/B70,"")</f>
-        <v>2.9942258192140577E-2</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
         <v>141</v>
+      </c>
+      <c r="B74" s="8">
+        <f>IFERROR(C62-B72,"")</f>
+        <v>60969.390195582528</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>142</v>
+      </c>
+      <c r="B75" s="18">
+        <f>IFERROR(B74/B71,"")</f>
+        <v>2.9916285670060123E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{58439CC7-F636-4EF3-B5B5-901BD02C3677}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{484FFEFE-D652-4748-8A0F-6C91B61F8B21}"/>
   </hyperlinks>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.5" footer="0.5"/>
-  <pageSetup scale="50" orientation="landscape" r:id="rId2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" r:id="rId2"/>
   <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2619 S Sepulveda OM and re-underwrite from it; move to OM-on-file section
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/02-2001-penmar-ave.xlsx
+++ b/files/02-2001-penmar-ave.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iniculete\LAAA-Deploys\onmarket\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3CF6438-C08C-47BD-AC5E-A50A5340BDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A43E3D39-CD3B-4215-8180-78064E182085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E2BABCE3-DF98-4F8E-954C-23F2036EA389}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0DCFCC4A-A33C-40CC-B566-BDC3096606E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="1" r:id="rId1"/>
@@ -195,7 +195,7 @@
     <t>Data pulled 9/17/2026 from LoopNet public listing + rent roll and expenses read from the listing broker's OM (RE/MAX, Taksa Investment Group, undated, rent roll May 2026)</t>
   </si>
   <si>
-    <t>NOTE: New listing 9/15/26, remodeled | OM: OM date not printed; latest move-in date on rent roll is 5/4/26 so the roll is mid-2026 or later.; Rent roll page text layer was scrambled; current rents read from the rendered page image. Unit-by-unit sum $37,286/mo vs OM total $37,283 ($3 rounding diff, within 1%); annual $447,401 per OM.; Current | OM: OM date not printed; latest move-in date on rent roll is 5/4/26 so the roll is mid-2026 or later.; Rent roll page text layer was scrambled; current rents read from the rendered page image. Unit-by-unit sum $37,286/mo vs OM total $37,283 ($3 rounding diff, within 1%); annual $447,401 per OM.; Current</t>
+    <t>NOTE: New listing 9/15/26, remodeled | OM: OM date not printed; latest move-in date on rent roll is 5/4/26 so the roll is mid-2026 or later.; Rent roll page text layer was scrambled; current rents read from the rendered page image. Unit-by-unit sum $37,286/mo vs OM total $37,283 ($3 rounding diff, within 1%); annual $447,401 per OM.; Current</t>
   </si>
   <si>
     <t>PROPERTY</t>
@@ -685,7 +685,7 @@
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C665A5E-A5CD-42B4-9617-4D7714C3C217}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47DC5BDB-3812-4A47-B0B8-9728A85FF9A8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -996,7 +996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE24FF7D-5CF0-45D4-80B2-C836386C6948}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65C588F0-59DD-4D44-9E7E-F9C00904AB6C}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1365,7 +1365,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA685BAD-5649-4B62-AEBC-769DA7D7186A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F006E58C-E3C5-42E2-9675-03565DA9589E}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -2264,7 +2264,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{484FFEFE-D652-4748-8A0F-6C91B61F8B21}"/>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{3D216DEB-7FE6-463D-B897-043889986EB1}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" r:id="rId2"/>

</xml_diff>